<commit_message>
release: faculty demo candidate 2026-09
</commit_message>
<xml_diff>
--- a/Code/templates/syllabus-import-template.xlsx
+++ b/Code/templates/syllabus-import-template.xlsx
@@ -13,9 +13,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reading List" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>course code</t>
+  </si>
+  <si>
+    <t>course name</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -417,200 +427,212 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>course designation</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>Core</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr" s="0">
         <is>
           <t>course types</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="inlineStr" s="0">
         <is>
           <t>Required</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="inlineStr" s="0">
         <is>
           <t>semester</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" t="inlineStr" s="0">
         <is>
           <t>HK1</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="inlineStr" s="0">
         <is>
           <t>language</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" t="inlineStr" s="0">
         <is>
           <t>English</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="inlineStr" s="0">
         <is>
           <t>relation</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="inlineStr" s="0">
         <is>
           <t>Undergraduate</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="inlineStr" s="0">
         <is>
           <t>teaching methods</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="inlineStr" s="0">
         <is>
           <t>Lecture, Lab</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="inlineStr" s="0">
         <is>
           <t>workload total</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" t="inlineStr" s="0">
         <is>
           <t>135</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr" s="0">
         <is>
           <t>workload contact</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" t="inlineStr" s="0">
         <is>
           <t>45</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr" s="0">
         <is>
           <t>workload private</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" t="inlineStr" s="0">
         <is>
           <t>90</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="inlineStr" s="0">
         <is>
           <t>prerequisites</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" t="inlineStr" s="0">
         <is>
           <t>None</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="inlineStr" s="0">
         <is>
           <t>objectives</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" t="inlineStr" s="0">
         <is>
           <t>Provide foundational knowledge</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="inlineStr" s="0">
         <is>
           <t>exam forms</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" t="inlineStr" s="0">
         <is>
           <t>Written exam</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="inlineStr" s="0">
         <is>
           <t>exam requirements</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" t="inlineStr" s="0">
         <is>
           <t>Minimum 5.0</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="inlineStr" s="0">
         <is>
           <t>rubrics</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" t="inlineStr" s="0">
         <is>
           <t>Course rubric</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="inlineStr" s="0">
         <is>
           <t>major</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" t="inlineStr" s="0">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B17" s="0"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B18" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -627,64 +649,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Description VN</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>Competency Level</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>Bloom Level</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>Order Index</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>CLO1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>Explain core concepts</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>Giải thích khái niệm cốt lõi</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr" s="0">
         <is>
           <t>KNOWLEDGE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr" s="0">
         <is>
           <t>UNDERSTAND</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="n" s="0">
         <v>1</v>
       </c>
     </row>
@@ -703,104 +725,104 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Week Number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Order In Week</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>Name VN</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>Teaching Hours</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>Lab Hours</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="0">
         <is>
           <t>Self Study Hours</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" t="inlineStr" s="0">
         <is>
           <t>Topic Type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" t="inlineStr" s="0">
         <is>
           <t>Teaching Method</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" t="inlineStr" s="0">
         <is>
           <t>Learning Activity</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" t="inlineStr" s="0">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="n" s="0">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="n" s="0">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>Introduction</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr" s="0">
         <is>
           <t>Giới thiệu</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" t="n" s="0">
         <v>3</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="n" s="0">
         <v>0</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="n" s="0">
         <v>6</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="inlineStr" s="0">
         <is>
           <t>LECTURE</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr" s="0">
         <is>
           <t>Lecture</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr" s="0">
         <is>
           <t>Discussion</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -817,68 +839,68 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Name VN</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Assessment Type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>Weight Percent</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>Min Score</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>Max Score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="0">
         <is>
           <t>Order Index</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>Thi cuối kỳ</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>FINAL_EXAM</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="n" s="0">
         <v>100</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" t="n" s="0">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="n" s="0">
         <v>10</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="n" s="0">
         <v>1</v>
       </c>
     </row>
@@ -897,98 +919,98 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Publisher</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>Edition</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>ISBN</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="0">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" t="inlineStr" s="0">
         <is>
           <t>Book Type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" t="inlineStr" s="0">
         <is>
           <t>Usage Type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" t="inlineStr" s="0">
         <is>
           <t>Order Index</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>Introduction to Computing</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>A. Author</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>Academic Press</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="n" s="0">
         <v>2026</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr" s="0">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr" s="0">
         <is>
           <t>9780000000000</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr" s="0"/>
+      <c r="H2" t="inlineStr" s="0">
         <is>
           <t>TEXTBOOK</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr" s="0">
         <is>
           <t>REQUIRED</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" t="n" s="0">
         <v>1</v>
       </c>
     </row>

</xml_diff>